<commit_message>
Updated version and data names
</commit_message>
<xml_diff>
--- a/Lake Trends.xlsx
+++ b/Lake Trends.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://officemgmtentserv-my.sharepoint.com/personal/jordon_henderson_owrb_ok_gov/Documents/Documents/Factsheets_HTML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="13_ncr:1_{AB8F8A81-B659-460C-97B1-4A36028393DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{546F70C8-066F-4A68-8D81-963E85BC223A}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="13_ncr:1_{AB8F8A81-B659-460C-97B1-4A36028393DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAB61BA7-7C8B-4B2D-AD0A-9AD1198CDCC7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45EE3177-148E-4463-BCC1-B47E3C070BBF}"/>
+    <workbookView xWindow="28680" yWindow="1395" windowWidth="29040" windowHeight="15720" xr2:uid="{45EE3177-148E-4463-BCC1-B47E3C070BBF}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL Info" sheetId="1" r:id="rId1"/>

</xml_diff>